<commit_message>
add new photos and update items
</commit_message>
<xml_diff>
--- a/items/items.xlsx
+++ b/items/items.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\listing-web\items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA165688-D8AE-4AB1-A109-7938CC224DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18EEE99-F5D5-4695-BBF8-95CBC30909F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3790" yWindow="1670" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Label</t>
   </si>
@@ -121,10 +121,22 @@
     <t>Chinese Cleaver</t>
   </si>
   <si>
-    <t>Stainless Steel Mixing Bowl</t>
-  </si>
-  <si>
     <t>Rice Cooker</t>
+  </si>
+  <si>
+    <t>About 79''/2m length and adjustable/scalable height</t>
+  </si>
+  <si>
+    <t>3 Stainless Steel Mixing Bowl</t>
+  </si>
+  <si>
+    <t>Almost new, bought from target</t>
+  </si>
+  <si>
+    <t>Hair Dryer</t>
+  </si>
+  <si>
+    <t>Not Dyson</t>
   </si>
 </sst>
 </file>
@@ -445,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="29.453125" bestFit="1" customWidth="1"/>
@@ -545,7 +557,7 @@
         <v>13</v>
       </c>
       <c r="C6">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -646,10 +658,13 @@
         <v>21</v>
       </c>
       <c r="C13">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D13">
         <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -660,7 +675,7 @@
         <v>22</v>
       </c>
       <c r="C14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -674,10 +689,13 @@
         <v>23</v>
       </c>
       <c r="C15">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="D15">
         <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -697,7 +715,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -711,7 +729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -725,7 +743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -739,7 +757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -753,7 +771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -767,12 +785,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C22">
         <v>8</v>
@@ -781,18 +799,35 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C23">
         <v>10</v>
       </c>
       <c r="D23">
         <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24">
+        <v>10</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>